<commit_message>
Incorporate verified Concentric AR2023 figures into benchmarks and deck
Gross margin 25.2% (2023) and expensed product development of MSEK 95
(2.3% of sales) replace earlier unverified estimates; pump-panel margin
statistics and the peer-margin scenario slide recalculated.

https://claude.ai/code/session_014jXqZEZtChXkgzZqCUB3kX
</commit_message>
<xml_diff>
--- a/competitor_gross_margin_benchmark.xlsx
+++ b/competitor_gross_margin_benchmark.xlsx
@@ -1001,27 +1001,25 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>not disclosed ('30%+' unverified)</t>
-        </is>
+          <t>2023 (last public)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>0.252</v>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MSEK 1,061</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes — IFRS cost-of-sales, company-reported (AR2023)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Operating margin 14.2% (16.7% in 2022) — 8x TBK's EBIT margin</t>
+          <t>2022: 26.3%. Op margin 14.2% (2023) vs 23.5% (2019, pre-EMP) — margin traded for electrification transition</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1236,7 @@
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>3. Pump peers bracket TBK: Hanon 9.1% below, Aisin ~12% just above, TPR ~22% well above. Concentric's 14.2% operating margin vs TBK's 1.7% EBIT margin is the starkest gap.</t>
+          <t>3. Pump peers (incl. Concentric, verified 25.2% per AR2023): Hanon 9.1% below, Aisin ~12% around TBK, TPR ~22% and Concentric 25.2% well above. Comparable pump-panel stats: average 17.0%, median 16.9%.</t>
         </is>
       </c>
     </row>

</xml_diff>